<commit_message>
Updated ITA model - 2025-09-16 23:56
</commit_message>
<xml_diff>
--- a/VerveStacks_ITA/SysSettings.xlsx
+++ b/VerveStacks_ITA/SysSettings.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\VerveStacks\assumptions\VerveStacks_ISO_template\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\vervestacks_models\VerveStacks_ITA\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1990339A-55DD-40A5-83CE-64097658B340}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BAC0DEE4-BA35-4396-8DEA-6055DF4D8335}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="system_settings" sheetId="1" r:id="rId1"/>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="546" uniqueCount="213">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="924" uniqueCount="339">
   <si>
     <t>~BookRegions_Map</t>
   </si>
@@ -52,9 +52,6 @@
     <t>~TimeSlices</t>
   </si>
   <si>
-    <t>GBL</t>
-  </si>
-  <si>
     <t>Season</t>
   </si>
   <si>
@@ -677,6 +674,387 @@
   </si>
   <si>
     <t>OIL</t>
+  </si>
+  <si>
+    <t>ITA</t>
+  </si>
+  <si>
+    <t>set</t>
+  </si>
+  <si>
+    <t>elc_spv_001</t>
+  </si>
+  <si>
+    <t>solar electricity generation in cluster -- 1</t>
+  </si>
+  <si>
+    <t>TWh</t>
+  </si>
+  <si>
+    <t>elc_spv_002</t>
+  </si>
+  <si>
+    <t>solar electricity generation in cluster -- 2</t>
+  </si>
+  <si>
+    <t>elc_spv_003</t>
+  </si>
+  <si>
+    <t>solar electricity generation in cluster -- 3</t>
+  </si>
+  <si>
+    <t>elc_spv_004</t>
+  </si>
+  <si>
+    <t>solar electricity generation in cluster -- 4</t>
+  </si>
+  <si>
+    <t>elc_spv_005</t>
+  </si>
+  <si>
+    <t>solar electricity generation in cluster -- 5</t>
+  </si>
+  <si>
+    <t>elc_spv_006</t>
+  </si>
+  <si>
+    <t>solar electricity generation in cluster -- 6</t>
+  </si>
+  <si>
+    <t>elc_spv_007</t>
+  </si>
+  <si>
+    <t>solar electricity generation in cluster -- 7</t>
+  </si>
+  <si>
+    <t>elc_spv_008</t>
+  </si>
+  <si>
+    <t>solar electricity generation in cluster -- 8</t>
+  </si>
+  <si>
+    <t>elc_spv_009</t>
+  </si>
+  <si>
+    <t>solar electricity generation in cluster -- 9</t>
+  </si>
+  <si>
+    <t>elc_spv_010</t>
+  </si>
+  <si>
+    <t>solar electricity generation in cluster -- 10</t>
+  </si>
+  <si>
+    <t>elc_spv_011</t>
+  </si>
+  <si>
+    <t>solar electricity generation in cluster -- 11</t>
+  </si>
+  <si>
+    <t>elc_spv_012</t>
+  </si>
+  <si>
+    <t>solar electricity generation in cluster -- 12</t>
+  </si>
+  <si>
+    <t>elc_spv_013</t>
+  </si>
+  <si>
+    <t>solar electricity generation in cluster -- 13</t>
+  </si>
+  <si>
+    <t>elc_spv_014</t>
+  </si>
+  <si>
+    <t>solar electricity generation in cluster -- 14</t>
+  </si>
+  <si>
+    <t>elc_spv_015</t>
+  </si>
+  <si>
+    <t>solar electricity generation in cluster -- 15</t>
+  </si>
+  <si>
+    <t>elc_spv_016</t>
+  </si>
+  <si>
+    <t>solar electricity generation in cluster -- 16</t>
+  </si>
+  <si>
+    <t>elc_spv_017</t>
+  </si>
+  <si>
+    <t>solar electricity generation in cluster -- 17</t>
+  </si>
+  <si>
+    <t>elc_spv_018</t>
+  </si>
+  <si>
+    <t>solar electricity generation in cluster -- 18</t>
+  </si>
+  <si>
+    <t>elc_spv_019</t>
+  </si>
+  <si>
+    <t>solar electricity generation in cluster -- 19</t>
+  </si>
+  <si>
+    <t>elc_spv_020</t>
+  </si>
+  <si>
+    <t>solar electricity generation in cluster -- 20</t>
+  </si>
+  <si>
+    <t>elc_spv_021</t>
+  </si>
+  <si>
+    <t>solar electricity generation in cluster -- 21</t>
+  </si>
+  <si>
+    <t>elc_spv_022</t>
+  </si>
+  <si>
+    <t>solar electricity generation in cluster -- 22</t>
+  </si>
+  <si>
+    <t>elc_spv_023</t>
+  </si>
+  <si>
+    <t>solar electricity generation in cluster -- 23</t>
+  </si>
+  <si>
+    <t>elc_spv_024</t>
+  </si>
+  <si>
+    <t>solar electricity generation in cluster -- 24</t>
+  </si>
+  <si>
+    <t>elc_wof_001</t>
+  </si>
+  <si>
+    <t>offwind electricity generation in cluster -- 1</t>
+  </si>
+  <si>
+    <t>elc_wof_002</t>
+  </si>
+  <si>
+    <t>offwind electricity generation in cluster -- 2</t>
+  </si>
+  <si>
+    <t>elc_wof_003</t>
+  </si>
+  <si>
+    <t>offwind electricity generation in cluster -- 3</t>
+  </si>
+  <si>
+    <t>elc_wof_004</t>
+  </si>
+  <si>
+    <t>offwind electricity generation in cluster -- 4</t>
+  </si>
+  <si>
+    <t>elc_wof_005</t>
+  </si>
+  <si>
+    <t>offwind electricity generation in cluster -- 5</t>
+  </si>
+  <si>
+    <t>elc_wof_006</t>
+  </si>
+  <si>
+    <t>offwind electricity generation in cluster -- 6</t>
+  </si>
+  <si>
+    <t>elc_wof_007</t>
+  </si>
+  <si>
+    <t>offwind electricity generation in cluster -- 7</t>
+  </si>
+  <si>
+    <t>elc_wof_008</t>
+  </si>
+  <si>
+    <t>offwind electricity generation in cluster -- 8</t>
+  </si>
+  <si>
+    <t>elc_wof_009</t>
+  </si>
+  <si>
+    <t>offwind electricity generation in cluster -- 9</t>
+  </si>
+  <si>
+    <t>elc_wof_010</t>
+  </si>
+  <si>
+    <t>offwind electricity generation in cluster -- 10</t>
+  </si>
+  <si>
+    <t>elc_wof_011</t>
+  </si>
+  <si>
+    <t>offwind electricity generation in cluster -- 11</t>
+  </si>
+  <si>
+    <t>elc_wof_012</t>
+  </si>
+  <si>
+    <t>offwind electricity generation in cluster -- 12</t>
+  </si>
+  <si>
+    <t>elc_wof_013</t>
+  </si>
+  <si>
+    <t>offwind electricity generation in cluster -- 13</t>
+  </si>
+  <si>
+    <t>elc_wof_014</t>
+  </si>
+  <si>
+    <t>offwind electricity generation in cluster -- 14</t>
+  </si>
+  <si>
+    <t>elc_wof_015</t>
+  </si>
+  <si>
+    <t>offwind electricity generation in cluster -- 15</t>
+  </si>
+  <si>
+    <t>elc_wof_016</t>
+  </si>
+  <si>
+    <t>offwind electricity generation in cluster -- 16</t>
+  </si>
+  <si>
+    <t>elc_wof_017</t>
+  </si>
+  <si>
+    <t>offwind electricity generation in cluster -- 17</t>
+  </si>
+  <si>
+    <t>elc_wof_018</t>
+  </si>
+  <si>
+    <t>offwind electricity generation in cluster -- 18</t>
+  </si>
+  <si>
+    <t>elc_wof_019</t>
+  </si>
+  <si>
+    <t>offwind electricity generation in cluster -- 19</t>
+  </si>
+  <si>
+    <t>elc_won_001</t>
+  </si>
+  <si>
+    <t>onshore wind electricity generation in cluster -- 1</t>
+  </si>
+  <si>
+    <t>elc_won_002</t>
+  </si>
+  <si>
+    <t>onshore wind electricity generation in cluster -- 2</t>
+  </si>
+  <si>
+    <t>elc_won_003</t>
+  </si>
+  <si>
+    <t>onshore wind electricity generation in cluster -- 3</t>
+  </si>
+  <si>
+    <t>elc_won_004</t>
+  </si>
+  <si>
+    <t>onshore wind electricity generation in cluster -- 4</t>
+  </si>
+  <si>
+    <t>elc_won_005</t>
+  </si>
+  <si>
+    <t>onshore wind electricity generation in cluster -- 5</t>
+  </si>
+  <si>
+    <t>elc_won_006</t>
+  </si>
+  <si>
+    <t>onshore wind electricity generation in cluster -- 6</t>
+  </si>
+  <si>
+    <t>elc_won_007</t>
+  </si>
+  <si>
+    <t>onshore wind electricity generation in cluster -- 7</t>
+  </si>
+  <si>
+    <t>elc_won_008</t>
+  </si>
+  <si>
+    <t>onshore wind electricity generation in cluster -- 8</t>
+  </si>
+  <si>
+    <t>elc_won_009</t>
+  </si>
+  <si>
+    <t>onshore wind electricity generation in cluster -- 9</t>
+  </si>
+  <si>
+    <t>elc_won_010</t>
+  </si>
+  <si>
+    <t>onshore wind electricity generation in cluster -- 10</t>
+  </si>
+  <si>
+    <t>elc_won_011</t>
+  </si>
+  <si>
+    <t>onshore wind electricity generation in cluster -- 11</t>
+  </si>
+  <si>
+    <t>elc_won_012</t>
+  </si>
+  <si>
+    <t>onshore wind electricity generation in cluster -- 12</t>
+  </si>
+  <si>
+    <t>elc_won_013</t>
+  </si>
+  <si>
+    <t>onshore wind electricity generation in cluster -- 13</t>
+  </si>
+  <si>
+    <t>elc_won_014</t>
+  </si>
+  <si>
+    <t>onshore wind electricity generation in cluster -- 14</t>
+  </si>
+  <si>
+    <t>elc_won_015</t>
+  </si>
+  <si>
+    <t>onshore wind electricity generation in cluster -- 15</t>
+  </si>
+  <si>
+    <t>elc_won_016</t>
+  </si>
+  <si>
+    <t>onshore wind electricity generation in cluster -- 16</t>
+  </si>
+  <si>
+    <t>elc_won_017</t>
+  </si>
+  <si>
+    <t>onshore wind electricity generation in cluster -- 17</t>
+  </si>
+  <si>
+    <t>elc_won_018</t>
+  </si>
+  <si>
+    <t>onshore wind electricity generation in cluster -- 18</t>
+  </si>
+  <si>
+    <t>elc_won_019</t>
+  </si>
+  <si>
+    <t>onshore wind electricity generation in cluster -- 19</t>
   </si>
 </sst>
 </file>
@@ -3053,35 +3431,35 @@
         <v>2</v>
       </c>
       <c r="F3" t="s">
+        <v>4</v>
+      </c>
+      <c r="G3" t="s">
         <v>5</v>
       </c>
-      <c r="G3" t="s">
+      <c r="H3" t="s">
         <v>6</v>
-      </c>
-      <c r="H3" t="s">
-        <v>7</v>
       </c>
     </row>
     <row r="4" spans="2:8">
       <c r="B4" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="C4" t="s">
-        <v>4</v>
+        <v>212</v>
       </c>
       <c r="F4" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="H4" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
     </row>
     <row r="5" spans="2:8">
       <c r="F5" t="s">
+        <v>37</v>
+      </c>
+      <c r="H5" t="s">
         <v>38</v>
-      </c>
-      <c r="H5" t="s">
-        <v>39</v>
       </c>
     </row>
   </sheetData>
@@ -3092,7 +3470,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B2F298A9-BCD9-4ABF-BE3B-9D1BDD3E7001}">
-  <dimension ref="B3:Q24"/>
+  <dimension ref="B3:R66"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <cols>
     <col min="2" max="2" width="11.19921875" bestFit="1" customWidth="1"/>
@@ -3105,9 +3483,9 @@
     <col min="9" max="9" width="12" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="3" spans="2:17" ht="17.649999999999999" thickBot="1">
+    <row r="3" spans="2:18" ht="17.649999999999999" thickBot="1">
       <c r="B3" s="3" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="C3" s="2"/>
       <c r="D3" s="2"/>
@@ -3117,304 +3495,1517 @@
       <c r="H3" s="1"/>
       <c r="I3" s="1"/>
       <c r="M3" s="3" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="N3" s="2"/>
       <c r="O3" s="2"/>
       <c r="P3" s="2"/>
       <c r="Q3" s="2"/>
     </row>
-    <row r="4" spans="2:17" ht="15" thickTop="1" thickBot="1">
+    <row r="4" spans="2:18" ht="15" thickTop="1" thickBot="1">
       <c r="B4" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="C4" s="5" t="s">
         <v>10</v>
       </c>
-      <c r="C4" s="5" t="s">
+      <c r="D4" s="5" t="s">
         <v>11</v>
       </c>
-      <c r="D4" s="5" t="s">
+      <c r="E4" s="5" t="s">
         <v>12</v>
       </c>
-      <c r="E4" s="5" t="s">
+      <c r="F4" s="5" t="s">
         <v>13</v>
       </c>
-      <c r="F4" s="5" t="s">
+      <c r="G4" s="5" t="s">
         <v>14</v>
       </c>
-      <c r="G4" s="5" t="s">
+      <c r="H4" s="5" t="s">
         <v>15</v>
       </c>
-      <c r="H4" s="5" t="s">
+      <c r="I4" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="I4" s="4" t="s">
+      <c r="M4" s="5" t="s">
+        <v>213</v>
+      </c>
+      <c r="N4" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="O4" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="P4" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="Q4" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="R4" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="5" spans="2:18">
+      <c r="B5" t="s">
         <v>17</v>
       </c>
-      <c r="M4" s="5"/>
-      <c r="N4" s="5"/>
-      <c r="O4" s="5"/>
-      <c r="P4" s="5"/>
-      <c r="Q4" s="5"/>
-    </row>
-    <row r="5" spans="2:17">
-      <c r="B5" t="s">
+      <c r="C5" t="s">
+        <v>19</v>
+      </c>
+      <c r="E5" t="s">
         <v>18</v>
       </c>
-      <c r="C5" t="s">
+      <c r="M5" t="s">
+        <v>17</v>
+      </c>
+      <c r="N5" t="s">
+        <v>214</v>
+      </c>
+      <c r="O5" t="s">
+        <v>215</v>
+      </c>
+      <c r="P5" t="s">
+        <v>25</v>
+      </c>
+      <c r="Q5" t="s">
+        <v>35</v>
+      </c>
+      <c r="R5" t="s">
+        <v>216</v>
+      </c>
+    </row>
+    <row r="6" spans="2:18">
+      <c r="B6" t="s">
+        <v>17</v>
+      </c>
+      <c r="C6" t="s">
+        <v>209</v>
+      </c>
+      <c r="E6" t="s">
+        <v>18</v>
+      </c>
+      <c r="M6" t="s">
+        <v>17</v>
+      </c>
+      <c r="N6" t="s">
+        <v>217</v>
+      </c>
+      <c r="O6" t="s">
+        <v>218</v>
+      </c>
+      <c r="P6" t="s">
+        <v>25</v>
+      </c>
+      <c r="Q6" t="s">
+        <v>35</v>
+      </c>
+      <c r="R6" t="s">
+        <v>216</v>
+      </c>
+    </row>
+    <row r="7" spans="2:18">
+      <c r="B7" t="s">
+        <v>17</v>
+      </c>
+      <c r="C7" t="s">
+        <v>210</v>
+      </c>
+      <c r="E7" t="s">
+        <v>18</v>
+      </c>
+      <c r="M7" t="s">
+        <v>17</v>
+      </c>
+      <c r="N7" t="s">
+        <v>219</v>
+      </c>
+      <c r="O7" t="s">
+        <v>220</v>
+      </c>
+      <c r="P7" t="s">
+        <v>25</v>
+      </c>
+      <c r="Q7" t="s">
+        <v>35</v>
+      </c>
+      <c r="R7" t="s">
+        <v>216</v>
+      </c>
+    </row>
+    <row r="8" spans="2:18">
+      <c r="B8" t="s">
+        <v>17</v>
+      </c>
+      <c r="C8" t="s">
+        <v>21</v>
+      </c>
+      <c r="E8" t="s">
+        <v>18</v>
+      </c>
+      <c r="M8" t="s">
+        <v>17</v>
+      </c>
+      <c r="N8" t="s">
+        <v>221</v>
+      </c>
+      <c r="O8" t="s">
+        <v>222</v>
+      </c>
+      <c r="P8" t="s">
+        <v>25</v>
+      </c>
+      <c r="Q8" t="s">
+        <v>35</v>
+      </c>
+      <c r="R8" t="s">
+        <v>216</v>
+      </c>
+    </row>
+    <row r="9" spans="2:18">
+      <c r="B9" t="s">
+        <v>17</v>
+      </c>
+      <c r="C9" t="s">
+        <v>22</v>
+      </c>
+      <c r="E9" t="s">
+        <v>18</v>
+      </c>
+      <c r="M9" t="s">
+        <v>17</v>
+      </c>
+      <c r="N9" t="s">
+        <v>223</v>
+      </c>
+      <c r="O9" t="s">
+        <v>224</v>
+      </c>
+      <c r="P9" t="s">
+        <v>25</v>
+      </c>
+      <c r="Q9" t="s">
+        <v>35</v>
+      </c>
+      <c r="R9" t="s">
+        <v>216</v>
+      </c>
+    </row>
+    <row r="10" spans="2:18">
+      <c r="B10" t="s">
+        <v>17</v>
+      </c>
+      <c r="C10" t="s">
         <v>20</v>
       </c>
-      <c r="E5" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="6" spans="2:17">
-      <c r="B6" t="s">
+      <c r="E10" t="s">
         <v>18</v>
       </c>
-      <c r="C6" t="s">
-        <v>210</v>
-      </c>
-      <c r="E6" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="7" spans="2:17">
-      <c r="B7" t="s">
+      <c r="M10" t="s">
+        <v>17</v>
+      </c>
+      <c r="N10" t="s">
+        <v>225</v>
+      </c>
+      <c r="O10" t="s">
+        <v>226</v>
+      </c>
+      <c r="P10" t="s">
+        <v>25</v>
+      </c>
+      <c r="Q10" t="s">
+        <v>35</v>
+      </c>
+      <c r="R10" t="s">
+        <v>216</v>
+      </c>
+    </row>
+    <row r="11" spans="2:18">
+      <c r="B11" t="s">
+        <v>17</v>
+      </c>
+      <c r="C11" t="s">
+        <v>23</v>
+      </c>
+      <c r="E11" t="s">
         <v>18</v>
       </c>
-      <c r="C7" t="s">
+      <c r="M11" t="s">
+        <v>17</v>
+      </c>
+      <c r="N11" t="s">
+        <v>227</v>
+      </c>
+      <c r="O11" t="s">
+        <v>228</v>
+      </c>
+      <c r="P11" t="s">
+        <v>25</v>
+      </c>
+      <c r="Q11" t="s">
+        <v>35</v>
+      </c>
+      <c r="R11" t="s">
+        <v>216</v>
+      </c>
+    </row>
+    <row r="12" spans="2:18">
+      <c r="B12" t="s">
+        <v>17</v>
+      </c>
+      <c r="C12" t="s">
         <v>211</v>
       </c>
-      <c r="E7" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="8" spans="2:17">
-      <c r="B8" t="s">
+      <c r="E12" t="s">
         <v>18</v>
       </c>
-      <c r="C8" t="s">
-        <v>22</v>
-      </c>
-      <c r="E8" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="9" spans="2:17">
-      <c r="B9" t="s">
+      <c r="M12" t="s">
+        <v>17</v>
+      </c>
+      <c r="N12" t="s">
+        <v>229</v>
+      </c>
+      <c r="O12" t="s">
+        <v>230</v>
+      </c>
+      <c r="P12" t="s">
+        <v>25</v>
+      </c>
+      <c r="Q12" t="s">
+        <v>35</v>
+      </c>
+      <c r="R12" t="s">
+        <v>216</v>
+      </c>
+    </row>
+    <row r="13" spans="2:18">
+      <c r="B13" t="s">
+        <v>17</v>
+      </c>
+      <c r="C13" t="s">
+        <v>24</v>
+      </c>
+      <c r="E13" t="s">
         <v>18</v>
       </c>
-      <c r="C9" t="s">
-        <v>23</v>
-      </c>
-      <c r="E9" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="10" spans="2:17">
-      <c r="B10" t="s">
+      <c r="M13" t="s">
+        <v>17</v>
+      </c>
+      <c r="N13" t="s">
+        <v>231</v>
+      </c>
+      <c r="O13" t="s">
+        <v>232</v>
+      </c>
+      <c r="P13" t="s">
+        <v>25</v>
+      </c>
+      <c r="Q13" t="s">
+        <v>35</v>
+      </c>
+      <c r="R13" t="s">
+        <v>216</v>
+      </c>
+    </row>
+    <row r="14" spans="2:18">
+      <c r="B14" t="s">
+        <v>17</v>
+      </c>
+      <c r="C14" t="s">
+        <v>205</v>
+      </c>
+      <c r="D14" t="s">
+        <v>207</v>
+      </c>
+      <c r="E14" t="s">
         <v>18</v>
       </c>
-      <c r="C10" t="s">
-        <v>21</v>
-      </c>
-      <c r="E10" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="11" spans="2:17">
-      <c r="B11" t="s">
+      <c r="M14" t="s">
+        <v>17</v>
+      </c>
+      <c r="N14" t="s">
+        <v>233</v>
+      </c>
+      <c r="O14" t="s">
+        <v>234</v>
+      </c>
+      <c r="P14" t="s">
+        <v>25</v>
+      </c>
+      <c r="Q14" t="s">
+        <v>35</v>
+      </c>
+      <c r="R14" t="s">
+        <v>216</v>
+      </c>
+    </row>
+    <row r="15" spans="2:18">
+      <c r="B15" t="s">
+        <v>17</v>
+      </c>
+      <c r="C15" t="s">
+        <v>206</v>
+      </c>
+      <c r="D15" t="s">
+        <v>208</v>
+      </c>
+      <c r="E15" t="s">
         <v>18</v>
       </c>
-      <c r="C11" t="s">
-        <v>24</v>
-      </c>
-      <c r="E11" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="12" spans="2:17">
-      <c r="B12" t="s">
+      <c r="M15" t="s">
+        <v>17</v>
+      </c>
+      <c r="N15" t="s">
+        <v>235</v>
+      </c>
+      <c r="O15" t="s">
+        <v>236</v>
+      </c>
+      <c r="P15" t="s">
+        <v>25</v>
+      </c>
+      <c r="Q15" t="s">
+        <v>35</v>
+      </c>
+      <c r="R15" t="s">
+        <v>216</v>
+      </c>
+    </row>
+    <row r="16" spans="2:18">
+      <c r="B16" t="s">
+        <v>17</v>
+      </c>
+      <c r="C16" t="s">
+        <v>25</v>
+      </c>
+      <c r="D16" t="s">
+        <v>30</v>
+      </c>
+      <c r="E16" t="s">
         <v>18</v>
       </c>
-      <c r="C12" t="s">
-        <v>212</v>
-      </c>
-      <c r="E12" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="13" spans="2:17">
-      <c r="B13" t="s">
+      <c r="F16" t="s">
+        <v>35</v>
+      </c>
+      <c r="G16" t="s">
+        <v>25</v>
+      </c>
+      <c r="I16" t="s">
+        <v>26</v>
+      </c>
+      <c r="M16" t="s">
+        <v>17</v>
+      </c>
+      <c r="N16" t="s">
+        <v>237</v>
+      </c>
+      <c r="O16" t="s">
+        <v>238</v>
+      </c>
+      <c r="P16" t="s">
+        <v>25</v>
+      </c>
+      <c r="Q16" t="s">
+        <v>35</v>
+      </c>
+      <c r="R16" t="s">
+        <v>216</v>
+      </c>
+    </row>
+    <row r="17" spans="2:18">
+      <c r="B17" t="s">
+        <v>34</v>
+      </c>
+      <c r="C17" t="s">
+        <v>203</v>
+      </c>
+      <c r="D17" t="s">
+        <v>204</v>
+      </c>
+      <c r="E17" t="s">
         <v>18</v>
       </c>
-      <c r="C13" t="s">
+      <c r="M17" t="s">
+        <v>17</v>
+      </c>
+      <c r="N17" t="s">
+        <v>239</v>
+      </c>
+      <c r="O17" t="s">
+        <v>240</v>
+      </c>
+      <c r="P17" t="s">
         <v>25</v>
       </c>
-      <c r="E13" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="14" spans="2:17">
-      <c r="B14" t="s">
+      <c r="Q17" t="s">
+        <v>35</v>
+      </c>
+      <c r="R17" t="s">
+        <v>216</v>
+      </c>
+    </row>
+    <row r="18" spans="2:18">
+      <c r="B18" t="s">
+        <v>34</v>
+      </c>
+      <c r="C18" t="s">
+        <v>27</v>
+      </c>
+      <c r="D18" t="s">
+        <v>31</v>
+      </c>
+      <c r="E18" t="s">
         <v>18</v>
       </c>
-      <c r="C14" t="s">
-        <v>206</v>
-      </c>
-      <c r="D14" t="s">
-        <v>208</v>
-      </c>
-      <c r="E14" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="15" spans="2:17">
-      <c r="B15" t="s">
+      <c r="M18" t="s">
+        <v>17</v>
+      </c>
+      <c r="N18" t="s">
+        <v>241</v>
+      </c>
+      <c r="O18" t="s">
+        <v>242</v>
+      </c>
+      <c r="P18" t="s">
+        <v>25</v>
+      </c>
+      <c r="Q18" t="s">
+        <v>35</v>
+      </c>
+      <c r="R18" t="s">
+        <v>216</v>
+      </c>
+    </row>
+    <row r="19" spans="2:18">
+      <c r="B19" t="s">
+        <v>34</v>
+      </c>
+      <c r="C19" t="s">
+        <v>28</v>
+      </c>
+      <c r="D19" t="s">
+        <v>32</v>
+      </c>
+      <c r="E19" t="s">
         <v>18</v>
       </c>
-      <c r="C15" t="s">
-        <v>207</v>
-      </c>
-      <c r="D15" t="s">
-        <v>209</v>
-      </c>
-      <c r="E15" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="16" spans="2:17">
-      <c r="B16" t="s">
+      <c r="M19" t="s">
+        <v>17</v>
+      </c>
+      <c r="N19" t="s">
+        <v>243</v>
+      </c>
+      <c r="O19" t="s">
+        <v>244</v>
+      </c>
+      <c r="P19" t="s">
+        <v>25</v>
+      </c>
+      <c r="Q19" t="s">
+        <v>35</v>
+      </c>
+      <c r="R19" t="s">
+        <v>216</v>
+      </c>
+    </row>
+    <row r="20" spans="2:18">
+      <c r="B20" t="s">
+        <v>34</v>
+      </c>
+      <c r="C20" t="s">
+        <v>29</v>
+      </c>
+      <c r="D20" t="s">
+        <v>33</v>
+      </c>
+      <c r="E20" t="s">
         <v>18</v>
       </c>
-      <c r="C16" t="s">
-        <v>26</v>
-      </c>
-      <c r="D16" t="s">
-        <v>31</v>
-      </c>
-      <c r="E16" t="s">
-        <v>19</v>
-      </c>
-      <c r="F16" t="s">
-        <v>36</v>
-      </c>
-      <c r="G16" t="s">
-        <v>26</v>
-      </c>
-      <c r="I16" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="17" spans="2:7">
-      <c r="B17" t="s">
+      <c r="M20" t="s">
+        <v>17</v>
+      </c>
+      <c r="N20" t="s">
+        <v>245</v>
+      </c>
+      <c r="O20" t="s">
+        <v>246</v>
+      </c>
+      <c r="P20" t="s">
+        <v>25</v>
+      </c>
+      <c r="Q20" t="s">
         <v>35</v>
       </c>
-      <c r="C17" t="s">
-        <v>204</v>
-      </c>
-      <c r="D17" t="s">
-        <v>205</v>
-      </c>
-      <c r="E17" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="18" spans="2:7">
-      <c r="B18" t="s">
+      <c r="R20" t="s">
+        <v>216</v>
+      </c>
+    </row>
+    <row r="21" spans="2:18">
+      <c r="B21" t="s">
+        <v>17</v>
+      </c>
+      <c r="C21" t="s">
+        <v>197</v>
+      </c>
+      <c r="D21" t="s">
+        <v>198</v>
+      </c>
+      <c r="E21" t="s">
+        <v>18</v>
+      </c>
+      <c r="F21" t="s">
         <v>35</v>
       </c>
-      <c r="C18" t="s">
-        <v>28</v>
-      </c>
-      <c r="D18" t="s">
-        <v>32</v>
-      </c>
-      <c r="E18" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="19" spans="2:7">
-      <c r="B19" t="s">
+      <c r="G21" t="s">
+        <v>25</v>
+      </c>
+      <c r="M21" t="s">
+        <v>17</v>
+      </c>
+      <c r="N21" t="s">
+        <v>247</v>
+      </c>
+      <c r="O21" t="s">
+        <v>248</v>
+      </c>
+      <c r="P21" t="s">
+        <v>25</v>
+      </c>
+      <c r="Q21" t="s">
         <v>35</v>
       </c>
-      <c r="C19" t="s">
-        <v>29</v>
-      </c>
-      <c r="D19" t="s">
-        <v>33</v>
-      </c>
-      <c r="E19" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="20" spans="2:7">
-      <c r="B20" t="s">
+      <c r="R21" t="s">
+        <v>216</v>
+      </c>
+    </row>
+    <row r="22" spans="2:18">
+      <c r="B22" t="s">
+        <v>193</v>
+      </c>
+      <c r="C22" t="s">
+        <v>194</v>
+      </c>
+      <c r="D22" t="s">
+        <v>195</v>
+      </c>
+      <c r="E22" t="s">
+        <v>196</v>
+      </c>
+      <c r="M22" t="s">
+        <v>17</v>
+      </c>
+      <c r="N22" t="s">
+        <v>249</v>
+      </c>
+      <c r="O22" t="s">
+        <v>250</v>
+      </c>
+      <c r="P22" t="s">
+        <v>25</v>
+      </c>
+      <c r="Q22" t="s">
         <v>35</v>
       </c>
-      <c r="C20" t="s">
-        <v>30</v>
-      </c>
-      <c r="D20" t="s">
-        <v>34</v>
-      </c>
-      <c r="E20" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="21" spans="2:7">
-      <c r="B21" t="s">
-        <v>18</v>
-      </c>
-      <c r="C21" t="s">
-        <v>198</v>
-      </c>
-      <c r="D21" t="s">
-        <v>199</v>
-      </c>
-      <c r="E21" t="s">
-        <v>19</v>
-      </c>
-      <c r="F21" t="s">
-        <v>36</v>
-      </c>
-      <c r="G21" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="22" spans="2:7">
-      <c r="B22" t="s">
-        <v>194</v>
-      </c>
-      <c r="C22" t="s">
-        <v>195</v>
-      </c>
-      <c r="D22" t="s">
+      <c r="R22" t="s">
+        <v>216</v>
+      </c>
+    </row>
+    <row r="23" spans="2:18">
+      <c r="B23" t="s">
+        <v>193</v>
+      </c>
+      <c r="C23" t="s">
+        <v>200</v>
+      </c>
+      <c r="E23" t="s">
         <v>196</v>
       </c>
-      <c r="E22" t="s">
-        <v>197</v>
-      </c>
-    </row>
-    <row r="23" spans="2:7">
-      <c r="B23" t="s">
-        <v>194</v>
-      </c>
-      <c r="C23" t="s">
+      <c r="M23" t="s">
+        <v>17</v>
+      </c>
+      <c r="N23" t="s">
+        <v>251</v>
+      </c>
+      <c r="O23" t="s">
+        <v>252</v>
+      </c>
+      <c r="P23" t="s">
+        <v>25</v>
+      </c>
+      <c r="Q23" t="s">
+        <v>35</v>
+      </c>
+      <c r="R23" t="s">
+        <v>216</v>
+      </c>
+    </row>
+    <row r="24" spans="2:18">
+      <c r="B24" t="s">
+        <v>193</v>
+      </c>
+      <c r="C24" t="s">
         <v>201</v>
       </c>
-      <c r="E23" t="s">
-        <v>197</v>
-      </c>
-    </row>
-    <row r="24" spans="2:7">
-      <c r="B24" t="s">
-        <v>194</v>
-      </c>
-      <c r="C24" t="s">
-        <v>202</v>
-      </c>
       <c r="E24" t="s">
-        <v>197</v>
+        <v>196</v>
+      </c>
+      <c r="M24" t="s">
+        <v>17</v>
+      </c>
+      <c r="N24" t="s">
+        <v>253</v>
+      </c>
+      <c r="O24" t="s">
+        <v>254</v>
+      </c>
+      <c r="P24" t="s">
+        <v>25</v>
+      </c>
+      <c r="Q24" t="s">
+        <v>35</v>
+      </c>
+      <c r="R24" t="s">
+        <v>216</v>
+      </c>
+    </row>
+    <row r="25" spans="2:18">
+      <c r="M25" t="s">
+        <v>17</v>
+      </c>
+      <c r="N25" t="s">
+        <v>255</v>
+      </c>
+      <c r="O25" t="s">
+        <v>256</v>
+      </c>
+      <c r="P25" t="s">
+        <v>25</v>
+      </c>
+      <c r="Q25" t="s">
+        <v>35</v>
+      </c>
+      <c r="R25" t="s">
+        <v>216</v>
+      </c>
+    </row>
+    <row r="26" spans="2:18">
+      <c r="M26" t="s">
+        <v>17</v>
+      </c>
+      <c r="N26" t="s">
+        <v>257</v>
+      </c>
+      <c r="O26" t="s">
+        <v>258</v>
+      </c>
+      <c r="P26" t="s">
+        <v>25</v>
+      </c>
+      <c r="Q26" t="s">
+        <v>35</v>
+      </c>
+      <c r="R26" t="s">
+        <v>216</v>
+      </c>
+    </row>
+    <row r="27" spans="2:18">
+      <c r="M27" t="s">
+        <v>17</v>
+      </c>
+      <c r="N27" t="s">
+        <v>259</v>
+      </c>
+      <c r="O27" t="s">
+        <v>260</v>
+      </c>
+      <c r="P27" t="s">
+        <v>25</v>
+      </c>
+      <c r="Q27" t="s">
+        <v>35</v>
+      </c>
+      <c r="R27" t="s">
+        <v>216</v>
+      </c>
+    </row>
+    <row r="28" spans="2:18">
+      <c r="M28" t="s">
+        <v>17</v>
+      </c>
+      <c r="N28" t="s">
+        <v>261</v>
+      </c>
+      <c r="O28" t="s">
+        <v>262</v>
+      </c>
+      <c r="P28" t="s">
+        <v>25</v>
+      </c>
+      <c r="Q28" t="s">
+        <v>35</v>
+      </c>
+      <c r="R28" t="s">
+        <v>216</v>
+      </c>
+    </row>
+    <row r="29" spans="2:18">
+      <c r="M29" t="s">
+        <v>17</v>
+      </c>
+      <c r="N29" t="s">
+        <v>263</v>
+      </c>
+      <c r="O29" t="s">
+        <v>264</v>
+      </c>
+      <c r="P29" t="s">
+        <v>25</v>
+      </c>
+      <c r="Q29" t="s">
+        <v>35</v>
+      </c>
+      <c r="R29" t="s">
+        <v>216</v>
+      </c>
+    </row>
+    <row r="30" spans="2:18">
+      <c r="M30" t="s">
+        <v>17</v>
+      </c>
+      <c r="N30" t="s">
+        <v>265</v>
+      </c>
+      <c r="O30" t="s">
+        <v>266</v>
+      </c>
+      <c r="P30" t="s">
+        <v>25</v>
+      </c>
+      <c r="Q30" t="s">
+        <v>35</v>
+      </c>
+      <c r="R30" t="s">
+        <v>216</v>
+      </c>
+    </row>
+    <row r="31" spans="2:18">
+      <c r="M31" t="s">
+        <v>17</v>
+      </c>
+      <c r="N31" t="s">
+        <v>267</v>
+      </c>
+      <c r="O31" t="s">
+        <v>268</v>
+      </c>
+      <c r="P31" t="s">
+        <v>25</v>
+      </c>
+      <c r="Q31" t="s">
+        <v>35</v>
+      </c>
+      <c r="R31" t="s">
+        <v>216</v>
+      </c>
+    </row>
+    <row r="32" spans="2:18">
+      <c r="M32" t="s">
+        <v>17</v>
+      </c>
+      <c r="N32" t="s">
+        <v>269</v>
+      </c>
+      <c r="O32" t="s">
+        <v>270</v>
+      </c>
+      <c r="P32" t="s">
+        <v>25</v>
+      </c>
+      <c r="Q32" t="s">
+        <v>35</v>
+      </c>
+      <c r="R32" t="s">
+        <v>216</v>
+      </c>
+    </row>
+    <row r="33" spans="13:18">
+      <c r="M33" t="s">
+        <v>17</v>
+      </c>
+      <c r="N33" t="s">
+        <v>271</v>
+      </c>
+      <c r="O33" t="s">
+        <v>272</v>
+      </c>
+      <c r="P33" t="s">
+        <v>25</v>
+      </c>
+      <c r="Q33" t="s">
+        <v>35</v>
+      </c>
+      <c r="R33" t="s">
+        <v>216</v>
+      </c>
+    </row>
+    <row r="34" spans="13:18">
+      <c r="M34" t="s">
+        <v>17</v>
+      </c>
+      <c r="N34" t="s">
+        <v>273</v>
+      </c>
+      <c r="O34" t="s">
+        <v>274</v>
+      </c>
+      <c r="P34" t="s">
+        <v>25</v>
+      </c>
+      <c r="Q34" t="s">
+        <v>35</v>
+      </c>
+      <c r="R34" t="s">
+        <v>216</v>
+      </c>
+    </row>
+    <row r="35" spans="13:18">
+      <c r="M35" t="s">
+        <v>17</v>
+      </c>
+      <c r="N35" t="s">
+        <v>275</v>
+      </c>
+      <c r="O35" t="s">
+        <v>276</v>
+      </c>
+      <c r="P35" t="s">
+        <v>25</v>
+      </c>
+      <c r="Q35" t="s">
+        <v>35</v>
+      </c>
+      <c r="R35" t="s">
+        <v>216</v>
+      </c>
+    </row>
+    <row r="36" spans="13:18">
+      <c r="M36" t="s">
+        <v>17</v>
+      </c>
+      <c r="N36" t="s">
+        <v>277</v>
+      </c>
+      <c r="O36" t="s">
+        <v>278</v>
+      </c>
+      <c r="P36" t="s">
+        <v>25</v>
+      </c>
+      <c r="Q36" t="s">
+        <v>35</v>
+      </c>
+      <c r="R36" t="s">
+        <v>216</v>
+      </c>
+    </row>
+    <row r="37" spans="13:18">
+      <c r="M37" t="s">
+        <v>17</v>
+      </c>
+      <c r="N37" t="s">
+        <v>279</v>
+      </c>
+      <c r="O37" t="s">
+        <v>280</v>
+      </c>
+      <c r="P37" t="s">
+        <v>25</v>
+      </c>
+      <c r="Q37" t="s">
+        <v>35</v>
+      </c>
+      <c r="R37" t="s">
+        <v>216</v>
+      </c>
+    </row>
+    <row r="38" spans="13:18">
+      <c r="M38" t="s">
+        <v>17</v>
+      </c>
+      <c r="N38" t="s">
+        <v>281</v>
+      </c>
+      <c r="O38" t="s">
+        <v>282</v>
+      </c>
+      <c r="P38" t="s">
+        <v>25</v>
+      </c>
+      <c r="Q38" t="s">
+        <v>35</v>
+      </c>
+      <c r="R38" t="s">
+        <v>216</v>
+      </c>
+    </row>
+    <row r="39" spans="13:18">
+      <c r="M39" t="s">
+        <v>17</v>
+      </c>
+      <c r="N39" t="s">
+        <v>283</v>
+      </c>
+      <c r="O39" t="s">
+        <v>284</v>
+      </c>
+      <c r="P39" t="s">
+        <v>25</v>
+      </c>
+      <c r="Q39" t="s">
+        <v>35</v>
+      </c>
+      <c r="R39" t="s">
+        <v>216</v>
+      </c>
+    </row>
+    <row r="40" spans="13:18">
+      <c r="M40" t="s">
+        <v>17</v>
+      </c>
+      <c r="N40" t="s">
+        <v>285</v>
+      </c>
+      <c r="O40" t="s">
+        <v>286</v>
+      </c>
+      <c r="P40" t="s">
+        <v>25</v>
+      </c>
+      <c r="Q40" t="s">
+        <v>35</v>
+      </c>
+      <c r="R40" t="s">
+        <v>216</v>
+      </c>
+    </row>
+    <row r="41" spans="13:18">
+      <c r="M41" t="s">
+        <v>17</v>
+      </c>
+      <c r="N41" t="s">
+        <v>287</v>
+      </c>
+      <c r="O41" t="s">
+        <v>288</v>
+      </c>
+      <c r="P41" t="s">
+        <v>25</v>
+      </c>
+      <c r="Q41" t="s">
+        <v>35</v>
+      </c>
+      <c r="R41" t="s">
+        <v>216</v>
+      </c>
+    </row>
+    <row r="42" spans="13:18">
+      <c r="M42" t="s">
+        <v>17</v>
+      </c>
+      <c r="N42" t="s">
+        <v>289</v>
+      </c>
+      <c r="O42" t="s">
+        <v>290</v>
+      </c>
+      <c r="P42" t="s">
+        <v>25</v>
+      </c>
+      <c r="Q42" t="s">
+        <v>35</v>
+      </c>
+      <c r="R42" t="s">
+        <v>216</v>
+      </c>
+    </row>
+    <row r="43" spans="13:18">
+      <c r="M43" t="s">
+        <v>17</v>
+      </c>
+      <c r="N43" t="s">
+        <v>291</v>
+      </c>
+      <c r="O43" t="s">
+        <v>292</v>
+      </c>
+      <c r="P43" t="s">
+        <v>25</v>
+      </c>
+      <c r="Q43" t="s">
+        <v>35</v>
+      </c>
+      <c r="R43" t="s">
+        <v>216</v>
+      </c>
+    </row>
+    <row r="44" spans="13:18">
+      <c r="M44" t="s">
+        <v>17</v>
+      </c>
+      <c r="N44" t="s">
+        <v>293</v>
+      </c>
+      <c r="O44" t="s">
+        <v>294</v>
+      </c>
+      <c r="P44" t="s">
+        <v>25</v>
+      </c>
+      <c r="Q44" t="s">
+        <v>35</v>
+      </c>
+      <c r="R44" t="s">
+        <v>216</v>
+      </c>
+    </row>
+    <row r="45" spans="13:18">
+      <c r="M45" t="s">
+        <v>17</v>
+      </c>
+      <c r="N45" t="s">
+        <v>295</v>
+      </c>
+      <c r="O45" t="s">
+        <v>296</v>
+      </c>
+      <c r="P45" t="s">
+        <v>25</v>
+      </c>
+      <c r="Q45" t="s">
+        <v>35</v>
+      </c>
+      <c r="R45" t="s">
+        <v>216</v>
+      </c>
+    </row>
+    <row r="46" spans="13:18">
+      <c r="M46" t="s">
+        <v>17</v>
+      </c>
+      <c r="N46" t="s">
+        <v>297</v>
+      </c>
+      <c r="O46" t="s">
+        <v>298</v>
+      </c>
+      <c r="P46" t="s">
+        <v>25</v>
+      </c>
+      <c r="Q46" t="s">
+        <v>35</v>
+      </c>
+      <c r="R46" t="s">
+        <v>216</v>
+      </c>
+    </row>
+    <row r="47" spans="13:18">
+      <c r="M47" t="s">
+        <v>17</v>
+      </c>
+      <c r="N47" t="s">
+        <v>299</v>
+      </c>
+      <c r="O47" t="s">
+        <v>300</v>
+      </c>
+      <c r="P47" t="s">
+        <v>25</v>
+      </c>
+      <c r="Q47" t="s">
+        <v>35</v>
+      </c>
+      <c r="R47" t="s">
+        <v>216</v>
+      </c>
+    </row>
+    <row r="48" spans="13:18">
+      <c r="M48" t="s">
+        <v>17</v>
+      </c>
+      <c r="N48" t="s">
+        <v>301</v>
+      </c>
+      <c r="O48" t="s">
+        <v>302</v>
+      </c>
+      <c r="P48" t="s">
+        <v>25</v>
+      </c>
+      <c r="Q48" t="s">
+        <v>35</v>
+      </c>
+      <c r="R48" t="s">
+        <v>216</v>
+      </c>
+    </row>
+    <row r="49" spans="13:18">
+      <c r="M49" t="s">
+        <v>17</v>
+      </c>
+      <c r="N49" t="s">
+        <v>303</v>
+      </c>
+      <c r="O49" t="s">
+        <v>304</v>
+      </c>
+      <c r="P49" t="s">
+        <v>25</v>
+      </c>
+      <c r="Q49" t="s">
+        <v>35</v>
+      </c>
+      <c r="R49" t="s">
+        <v>216</v>
+      </c>
+    </row>
+    <row r="50" spans="13:18">
+      <c r="M50" t="s">
+        <v>17</v>
+      </c>
+      <c r="N50" t="s">
+        <v>305</v>
+      </c>
+      <c r="O50" t="s">
+        <v>306</v>
+      </c>
+      <c r="P50" t="s">
+        <v>25</v>
+      </c>
+      <c r="Q50" t="s">
+        <v>35</v>
+      </c>
+      <c r="R50" t="s">
+        <v>216</v>
+      </c>
+    </row>
+    <row r="51" spans="13:18">
+      <c r="M51" t="s">
+        <v>17</v>
+      </c>
+      <c r="N51" t="s">
+        <v>307</v>
+      </c>
+      <c r="O51" t="s">
+        <v>308</v>
+      </c>
+      <c r="P51" t="s">
+        <v>25</v>
+      </c>
+      <c r="Q51" t="s">
+        <v>35</v>
+      </c>
+      <c r="R51" t="s">
+        <v>216</v>
+      </c>
+    </row>
+    <row r="52" spans="13:18">
+      <c r="M52" t="s">
+        <v>17</v>
+      </c>
+      <c r="N52" t="s">
+        <v>309</v>
+      </c>
+      <c r="O52" t="s">
+        <v>310</v>
+      </c>
+      <c r="P52" t="s">
+        <v>25</v>
+      </c>
+      <c r="Q52" t="s">
+        <v>35</v>
+      </c>
+      <c r="R52" t="s">
+        <v>216</v>
+      </c>
+    </row>
+    <row r="53" spans="13:18">
+      <c r="M53" t="s">
+        <v>17</v>
+      </c>
+      <c r="N53" t="s">
+        <v>311</v>
+      </c>
+      <c r="O53" t="s">
+        <v>312</v>
+      </c>
+      <c r="P53" t="s">
+        <v>25</v>
+      </c>
+      <c r="Q53" t="s">
+        <v>35</v>
+      </c>
+      <c r="R53" t="s">
+        <v>216</v>
+      </c>
+    </row>
+    <row r="54" spans="13:18">
+      <c r="M54" t="s">
+        <v>17</v>
+      </c>
+      <c r="N54" t="s">
+        <v>313</v>
+      </c>
+      <c r="O54" t="s">
+        <v>314</v>
+      </c>
+      <c r="P54" t="s">
+        <v>25</v>
+      </c>
+      <c r="Q54" t="s">
+        <v>35</v>
+      </c>
+      <c r="R54" t="s">
+        <v>216</v>
+      </c>
+    </row>
+    <row r="55" spans="13:18">
+      <c r="M55" t="s">
+        <v>17</v>
+      </c>
+      <c r="N55" t="s">
+        <v>315</v>
+      </c>
+      <c r="O55" t="s">
+        <v>316</v>
+      </c>
+      <c r="P55" t="s">
+        <v>25</v>
+      </c>
+      <c r="Q55" t="s">
+        <v>35</v>
+      </c>
+      <c r="R55" t="s">
+        <v>216</v>
+      </c>
+    </row>
+    <row r="56" spans="13:18">
+      <c r="M56" t="s">
+        <v>17</v>
+      </c>
+      <c r="N56" t="s">
+        <v>317</v>
+      </c>
+      <c r="O56" t="s">
+        <v>318</v>
+      </c>
+      <c r="P56" t="s">
+        <v>25</v>
+      </c>
+      <c r="Q56" t="s">
+        <v>35</v>
+      </c>
+      <c r="R56" t="s">
+        <v>216</v>
+      </c>
+    </row>
+    <row r="57" spans="13:18">
+      <c r="M57" t="s">
+        <v>17</v>
+      </c>
+      <c r="N57" t="s">
+        <v>319</v>
+      </c>
+      <c r="O57" t="s">
+        <v>320</v>
+      </c>
+      <c r="P57" t="s">
+        <v>25</v>
+      </c>
+      <c r="Q57" t="s">
+        <v>35</v>
+      </c>
+      <c r="R57" t="s">
+        <v>216</v>
+      </c>
+    </row>
+    <row r="58" spans="13:18">
+      <c r="M58" t="s">
+        <v>17</v>
+      </c>
+      <c r="N58" t="s">
+        <v>321</v>
+      </c>
+      <c r="O58" t="s">
+        <v>322</v>
+      </c>
+      <c r="P58" t="s">
+        <v>25</v>
+      </c>
+      <c r="Q58" t="s">
+        <v>35</v>
+      </c>
+      <c r="R58" t="s">
+        <v>216</v>
+      </c>
+    </row>
+    <row r="59" spans="13:18">
+      <c r="M59" t="s">
+        <v>17</v>
+      </c>
+      <c r="N59" t="s">
+        <v>323</v>
+      </c>
+      <c r="O59" t="s">
+        <v>324</v>
+      </c>
+      <c r="P59" t="s">
+        <v>25</v>
+      </c>
+      <c r="Q59" t="s">
+        <v>35</v>
+      </c>
+      <c r="R59" t="s">
+        <v>216</v>
+      </c>
+    </row>
+    <row r="60" spans="13:18">
+      <c r="M60" t="s">
+        <v>17</v>
+      </c>
+      <c r="N60" t="s">
+        <v>325</v>
+      </c>
+      <c r="O60" t="s">
+        <v>326</v>
+      </c>
+      <c r="P60" t="s">
+        <v>25</v>
+      </c>
+      <c r="Q60" t="s">
+        <v>35</v>
+      </c>
+      <c r="R60" t="s">
+        <v>216</v>
+      </c>
+    </row>
+    <row r="61" spans="13:18">
+      <c r="M61" t="s">
+        <v>17</v>
+      </c>
+      <c r="N61" t="s">
+        <v>327</v>
+      </c>
+      <c r="O61" t="s">
+        <v>328</v>
+      </c>
+      <c r="P61" t="s">
+        <v>25</v>
+      </c>
+      <c r="Q61" t="s">
+        <v>35</v>
+      </c>
+      <c r="R61" t="s">
+        <v>216</v>
+      </c>
+    </row>
+    <row r="62" spans="13:18">
+      <c r="M62" t="s">
+        <v>17</v>
+      </c>
+      <c r="N62" t="s">
+        <v>329</v>
+      </c>
+      <c r="O62" t="s">
+        <v>330</v>
+      </c>
+      <c r="P62" t="s">
+        <v>25</v>
+      </c>
+      <c r="Q62" t="s">
+        <v>35</v>
+      </c>
+      <c r="R62" t="s">
+        <v>216</v>
+      </c>
+    </row>
+    <row r="63" spans="13:18">
+      <c r="M63" t="s">
+        <v>17</v>
+      </c>
+      <c r="N63" t="s">
+        <v>331</v>
+      </c>
+      <c r="O63" t="s">
+        <v>332</v>
+      </c>
+      <c r="P63" t="s">
+        <v>25</v>
+      </c>
+      <c r="Q63" t="s">
+        <v>35</v>
+      </c>
+      <c r="R63" t="s">
+        <v>216</v>
+      </c>
+    </row>
+    <row r="64" spans="13:18">
+      <c r="M64" t="s">
+        <v>17</v>
+      </c>
+      <c r="N64" t="s">
+        <v>333</v>
+      </c>
+      <c r="O64" t="s">
+        <v>334</v>
+      </c>
+      <c r="P64" t="s">
+        <v>25</v>
+      </c>
+      <c r="Q64" t="s">
+        <v>35</v>
+      </c>
+      <c r="R64" t="s">
+        <v>216</v>
+      </c>
+    </row>
+    <row r="65" spans="13:18">
+      <c r="M65" t="s">
+        <v>17</v>
+      </c>
+      <c r="N65" t="s">
+        <v>335</v>
+      </c>
+      <c r="O65" t="s">
+        <v>336</v>
+      </c>
+      <c r="P65" t="s">
+        <v>25</v>
+      </c>
+      <c r="Q65" t="s">
+        <v>35</v>
+      </c>
+      <c r="R65" t="s">
+        <v>216</v>
+      </c>
+    </row>
+    <row r="66" spans="13:18">
+      <c r="M66" t="s">
+        <v>17</v>
+      </c>
+      <c r="N66" t="s">
+        <v>337</v>
+      </c>
+      <c r="O66" t="s">
+        <v>338</v>
+      </c>
+      <c r="P66" t="s">
+        <v>25</v>
+      </c>
+      <c r="Q66" t="s">
+        <v>35</v>
+      </c>
+      <c r="R66" t="s">
+        <v>216</v>
       </c>
     </row>
   </sheetData>
@@ -3441,7 +5032,7 @@
   <sheetData>
     <row r="3" spans="2:7">
       <c r="B3" s="6" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
     </row>
     <row r="4" spans="2:7">
@@ -3451,28 +5042,28 @@
     </row>
     <row r="7" spans="2:7">
       <c r="B7" s="6" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
     </row>
     <row r="8" spans="2:7">
       <c r="B8" s="6" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
     </row>
     <row r="11" spans="2:7">
       <c r="B11" s="6" t="s">
+        <v>43</v>
+      </c>
+      <c r="D11" s="6" t="s">
         <v>44</v>
-      </c>
-      <c r="D11" s="6" t="s">
-        <v>45</v>
       </c>
     </row>
     <row r="12" spans="2:7" ht="14.25">
       <c r="B12" s="7" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D12" s="8" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="E12" s="8" t="str">
         <f>"msy"&amp;COUNT(E14:E46)&amp;"_"&amp;MAX(E14:E46)</f>
@@ -3492,7 +5083,7 @@
         <v>1</v>
       </c>
       <c r="D13" s="6" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
     </row>
     <row r="14" spans="2:7" ht="14.25">
@@ -3500,7 +5091,7 @@
         <v>5</v>
       </c>
       <c r="D14" s="6" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="E14" s="6">
         <f t="shared" ref="E14:G14" si="1">$B$4</f>
@@ -3520,7 +5111,7 @@
         <v>5</v>
       </c>
       <c r="D15" s="6" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="E15" s="6">
         <f>E14+3</f>
@@ -3540,7 +5131,7 @@
         <v>10</v>
       </c>
       <c r="D16" s="6" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="E16" s="6">
         <f>E15+5</f>
@@ -3560,7 +5151,7 @@
         <v>10</v>
       </c>
       <c r="D17" s="6" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="E17" s="6">
         <f t="shared" ref="E17:E20" si="2">E16+5</f>
@@ -3580,7 +5171,7 @@
         <v>10</v>
       </c>
       <c r="D18" s="6" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="E18" s="6">
         <f t="shared" si="2"/>
@@ -3600,7 +5191,7 @@
         <v>10</v>
       </c>
       <c r="D19" s="6" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="E19" s="6">
         <f t="shared" si="2"/>
@@ -3616,7 +5207,7 @@
         <v>10</v>
       </c>
       <c r="D20" s="6" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="E20" s="6">
         <f t="shared" si="2"/>
@@ -3628,7 +5219,7 @@
         <v>10</v>
       </c>
       <c r="D21" s="6" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
     </row>
     <row r="22" spans="2:7" ht="14.25">
@@ -3636,7 +5227,7 @@
         <v>10</v>
       </c>
       <c r="D22" s="6" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
     </row>
     <row r="23" spans="2:7" ht="14.25">
@@ -3644,7 +5235,7 @@
         <v>10</v>
       </c>
       <c r="D23" s="6" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
     </row>
     <row r="24" spans="2:7" ht="14.25">
@@ -3652,37 +5243,37 @@
         <v>10</v>
       </c>
       <c r="D24" s="6" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
     </row>
     <row r="25" spans="2:7" ht="14.25">
       <c r="B25" s="9"/>
       <c r="D25" s="6" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
     </row>
     <row r="26" spans="2:7" ht="14.25">
       <c r="B26" s="9"/>
       <c r="D26" s="6" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
     </row>
     <row r="27" spans="2:7" ht="14.25">
       <c r="B27" s="9"/>
       <c r="D27" s="6" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
     </row>
     <row r="28" spans="2:7" ht="14.25">
       <c r="B28" s="9"/>
       <c r="D28" s="6" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
     </row>
     <row r="29" spans="2:7" ht="14.25">
       <c r="B29" s="9"/>
       <c r="D29" s="6" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
     </row>
     <row r="30" spans="2:7" ht="14.25">
@@ -3751,7 +5342,7 @@
     </row>
     <row r="4" spans="2:12">
       <c r="B4" s="14" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="G4" s="14"/>
       <c r="H4" s="14"/>
@@ -3759,42 +5350,42 @@
     </row>
     <row r="5" spans="2:12">
       <c r="B5" s="15" t="s">
+        <v>49</v>
+      </c>
+      <c r="C5" s="15" t="s">
         <v>50</v>
       </c>
-      <c r="C5" s="15" t="s">
+      <c r="D5" s="15" t="s">
         <v>51</v>
       </c>
-      <c r="D5" s="15" t="s">
+      <c r="E5" s="15" t="s">
         <v>52</v>
       </c>
-      <c r="E5" s="15" t="s">
+      <c r="F5" s="15" t="s">
         <v>53</v>
       </c>
-      <c r="F5" s="15" t="s">
+      <c r="G5" s="15" t="s">
         <v>54</v>
       </c>
-      <c r="G5" s="15" t="s">
+      <c r="H5" s="15" t="s">
         <v>55</v>
       </c>
-      <c r="H5" s="15" t="s">
+      <c r="I5" s="15" t="s">
         <v>56</v>
       </c>
-      <c r="I5" s="15" t="s">
+      <c r="J5" s="15" t="s">
         <v>57</v>
       </c>
-      <c r="J5" s="15" t="s">
+      <c r="K5" s="15" t="s">
         <v>58</v>
       </c>
-      <c r="K5" s="15" t="s">
+      <c r="L5" s="15" t="s">
         <v>59</v>
-      </c>
-      <c r="L5" s="15" t="s">
-        <v>60</v>
       </c>
     </row>
     <row r="6" spans="2:12">
       <c r="D6" s="11" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="E6" s="11">
         <v>0</v>
@@ -3805,7 +5396,7 @@
     </row>
     <row r="7" spans="2:12">
       <c r="D7" s="11" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="E7" s="11">
         <v>0</v>
@@ -3816,7 +5407,7 @@
     </row>
     <row r="8" spans="2:12">
       <c r="D8" s="11" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="E8" s="11">
         <v>0</v>
@@ -3827,7 +5418,7 @@
     </row>
     <row r="9" spans="2:12">
       <c r="D9" s="11" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="E9" s="11">
         <v>0</v>
@@ -3838,7 +5429,7 @@
     </row>
     <row r="10" spans="2:12">
       <c r="D10" s="11" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="E10" s="11">
         <v>0</v>
@@ -3849,7 +5440,7 @@
     </row>
     <row r="13" spans="2:12">
       <c r="B13" s="14" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="G13" s="14"/>
       <c r="H13" s="14"/>
@@ -3857,50 +5448,50 @@
     </row>
     <row r="14" spans="2:12">
       <c r="B14" s="15" t="s">
+        <v>49</v>
+      </c>
+      <c r="C14" s="15" t="s">
         <v>50</v>
       </c>
-      <c r="C14" s="15" t="s">
+      <c r="D14" s="15" t="s">
         <v>51</v>
       </c>
-      <c r="D14" s="15" t="s">
-        <v>52</v>
-      </c>
       <c r="E14" s="15" t="s">
+        <v>64</v>
+      </c>
+      <c r="F14" s="15" t="s">
+        <v>53</v>
+      </c>
+      <c r="G14" s="15" t="s">
         <v>65</v>
       </c>
-      <c r="F14" s="15" t="s">
-        <v>54</v>
-      </c>
-      <c r="G14" s="15" t="s">
-        <v>66</v>
-      </c>
       <c r="H14" s="15" t="s">
+        <v>55</v>
+      </c>
+      <c r="I14" s="15" t="s">
         <v>56</v>
-      </c>
-      <c r="I14" s="15" t="s">
-        <v>57</v>
       </c>
     </row>
     <row r="15" spans="2:12">
       <c r="D15" s="11" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="F15" s="11">
         <v>2222</v>
       </c>
       <c r="G15" s="11" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
     </row>
     <row r="16" spans="2:12">
       <c r="D16" s="11" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="F16" s="11">
         <v>8888</v>
       </c>
       <c r="G16" s="11" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
     </row>
     <row r="17" spans="2:14" ht="12.75">
@@ -4297,13 +5888,13 @@
     <row r="2" spans="1:14" ht="17.649999999999999" thickBot="1">
       <c r="A2" s="13"/>
       <c r="B2" s="20" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="E2" s="20" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="L2" s="20" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="M2" s="6"/>
       <c r="N2" s="6"/>
@@ -4311,56 +5902,56 @@
     <row r="3" spans="1:14" ht="15" thickTop="1" thickBot="1">
       <c r="A3" s="13"/>
       <c r="B3" s="4" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="E3" s="4" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="F3" s="4" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="G3" s="4" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="H3" s="4" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="I3" s="4">
         <v>2022</v>
       </c>
       <c r="J3" s="4" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="L3" s="4" t="s">
+        <v>80</v>
+      </c>
+      <c r="M3" s="4" t="s">
         <v>81</v>
       </c>
-      <c r="M3" s="4" t="s">
+      <c r="N3" s="4" t="s">
         <v>82</v>
-      </c>
-      <c r="N3" s="4" t="s">
-        <v>83</v>
       </c>
     </row>
     <row r="4" spans="1:14" ht="13.15">
       <c r="A4" s="13"/>
       <c r="B4" s="19" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="C4" s="6"/>
       <c r="F4" s="11" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="I4" s="11">
         <v>0.05</v>
       </c>
       <c r="J4" s="11" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="L4" s="6" t="s">
+        <v>84</v>
+      </c>
+      <c r="M4" s="6" t="s">
         <v>85</v>
-      </c>
-      <c r="M4" s="6" t="s">
-        <v>86</v>
       </c>
       <c r="N4" s="6">
         <v>1055.55</v>
@@ -4369,25 +5960,25 @@
     <row r="5" spans="1:14" ht="13.15">
       <c r="A5" s="13"/>
       <c r="B5" s="19" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="E5" s="11" t="s">
+        <v>186</v>
+      </c>
+      <c r="F5" s="11" t="s">
         <v>187</v>
-      </c>
-      <c r="F5" s="11" t="s">
-        <v>188</v>
       </c>
       <c r="I5" s="11">
         <v>1</v>
       </c>
       <c r="J5" s="11" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="L5" s="6" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="M5" s="6" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="N5" s="6">
         <v>3.6</v>
@@ -4396,19 +5987,19 @@
     <row r="6" spans="1:14" ht="13.15">
       <c r="A6" s="13"/>
       <c r="B6" s="19" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="F6" s="11" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="I6" s="11">
         <v>2025</v>
       </c>
       <c r="L6" s="6" t="s">
+        <v>89</v>
+      </c>
+      <c r="M6" s="6" t="s">
         <v>90</v>
-      </c>
-      <c r="M6" s="6" t="s">
-        <v>91</v>
       </c>
       <c r="N6" s="6">
         <v>1000</v>
@@ -4417,19 +6008,19 @@
     <row r="7" spans="1:14" ht="13.15">
       <c r="A7" s="13"/>
       <c r="B7" s="19" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="F7" s="11" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="I7" s="11">
         <v>1</v>
       </c>
       <c r="L7" s="6" t="s">
+        <v>92</v>
+      </c>
+      <c r="M7" s="6" t="s">
         <v>93</v>
-      </c>
-      <c r="M7" s="6" t="s">
-        <v>94</v>
       </c>
       <c r="N7" s="6">
         <v>1000</v>
@@ -4438,25 +6029,25 @@
     <row r="8" spans="1:14" ht="13.15">
       <c r="A8" s="13"/>
       <c r="B8" s="19" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="F8" s="11" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="G8" s="11" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="H8" s="11" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="I8" s="11">
         <v>2.2201</v>
       </c>
       <c r="L8" s="6" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="M8" s="6" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="N8" s="6">
         <v>1.05555</v>
@@ -4465,25 +6056,25 @@
     <row r="9" spans="1:14" ht="13.15">
       <c r="A9" s="13"/>
       <c r="B9" s="19" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="F9" s="11" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="G9" s="11" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="H9" s="11" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="I9" s="11">
         <v>2.1427</v>
       </c>
       <c r="L9" s="6" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="M9" s="6" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="N9" s="6">
         <v>4.1868000000000002E-2</v>
@@ -4492,25 +6083,25 @@
     <row r="10" spans="1:14" ht="13.15">
       <c r="A10" s="13"/>
       <c r="B10" s="19" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="F10" s="11" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="G10" s="11" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="H10" s="11" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="I10" s="11">
         <v>2.077</v>
       </c>
       <c r="L10" s="6" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="M10" s="6" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="N10" s="6">
         <v>41.868000000000002</v>
@@ -4519,25 +6110,25 @@
     <row r="11" spans="1:14" ht="13.15">
       <c r="A11" s="13"/>
       <c r="B11" s="19" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="F11" s="11" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="G11" s="11" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="H11" s="11" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="I11" s="11">
         <v>2.0358000000000001</v>
       </c>
       <c r="L11" s="6" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="M11" s="6" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="N11" s="6">
         <v>3.5999999999999999E-3</v>
@@ -4546,25 +6137,25 @@
     <row r="12" spans="1:14" ht="13.15">
       <c r="A12" s="13"/>
       <c r="B12" s="19" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="F12" s="11" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="G12" s="11" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="H12" s="11" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="I12" s="11">
         <v>1.9870000000000001</v>
       </c>
       <c r="L12" s="6" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="M12" s="6" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="N12" s="6">
         <v>1000000</v>
@@ -4573,25 +6164,25 @@
     <row r="13" spans="1:14" ht="13.15">
       <c r="A13" s="13"/>
       <c r="B13" s="19" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="F13" s="11" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="G13" s="11" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="H13" s="11" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="I13" s="11">
         <v>1.9192</v>
       </c>
       <c r="L13" s="6" t="s">
+        <v>105</v>
+      </c>
+      <c r="M13" s="6" t="s">
         <v>106</v>
-      </c>
-      <c r="M13" s="6" t="s">
-        <v>107</v>
       </c>
       <c r="N13" s="6">
         <v>1000</v>
@@ -4600,25 +6191,25 @@
     <row r="14" spans="1:14" ht="13.15">
       <c r="A14" s="13"/>
       <c r="B14" s="19" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="F14" s="11" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="G14" s="11" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="H14" s="11" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="I14" s="11">
         <v>1.8468</v>
       </c>
       <c r="L14" s="6" t="s">
+        <v>108</v>
+      </c>
+      <c r="M14" s="6" t="s">
         <v>109</v>
-      </c>
-      <c r="M14" s="6" t="s">
-        <v>110</v>
       </c>
       <c r="N14" s="6">
         <v>5.8615199999999996</v>
@@ -4627,25 +6218,25 @@
     <row r="15" spans="1:14" ht="13.15">
       <c r="A15" s="13"/>
       <c r="B15" s="19" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="F15" s="11" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="G15" s="11" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="H15" s="11" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="I15" s="11">
         <v>1.7799</v>
       </c>
       <c r="L15" s="6" t="s">
+        <v>111</v>
+      </c>
+      <c r="M15" s="6" t="s">
         <v>112</v>
-      </c>
-      <c r="M15" s="6" t="s">
-        <v>113</v>
       </c>
       <c r="N15" s="6">
         <v>1E-3</v>
@@ -4654,25 +6245,25 @@
     <row r="16" spans="1:14" ht="13.15">
       <c r="A16" s="13"/>
       <c r="B16" s="19" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="F16" s="11" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="G16" s="11" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="H16" s="11" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="I16" s="11">
         <v>1.722</v>
       </c>
       <c r="L16" s="6" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="M16" s="6" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="N16" s="6">
         <v>1000</v>
@@ -4681,25 +6272,25 @@
     <row r="17" spans="1:14" ht="13.15">
       <c r="A17" s="13"/>
       <c r="B17" s="19" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="F17" s="11" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="G17" s="11" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="H17" s="11" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="I17" s="11">
         <v>1.6836</v>
       </c>
       <c r="L17" s="6" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="M17" s="6" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="N17" s="6">
         <v>37.68</v>
@@ -4707,25 +6298,25 @@
     </row>
     <row r="18" spans="1:14" ht="13.15">
       <c r="B18" s="19" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="F18" s="11" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="G18" s="11" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="H18" s="11" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="I18" s="11">
         <v>1.6446000000000001</v>
       </c>
       <c r="L18" s="6" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="M18" s="6" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="N18" s="6">
         <v>2139.4548</v>
@@ -4733,25 +6324,25 @@
     </row>
     <row r="19" spans="1:14" ht="13.15">
       <c r="B19" s="19" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="F19" s="11" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="G19" s="11" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="H19" s="11" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="I19" s="11">
         <v>1.6102000000000001</v>
       </c>
       <c r="L19" s="6" t="s">
+        <v>120</v>
+      </c>
+      <c r="M19" s="6" t="s">
         <v>121</v>
-      </c>
-      <c r="M19" s="6" t="s">
-        <v>122</v>
       </c>
       <c r="N19" s="6">
         <v>2.78</v>
@@ -4759,25 +6350,25 @@
     </row>
     <row r="20" spans="1:14" ht="13.15">
       <c r="B20" s="19" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="F20" s="11" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="G20" s="11" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="H20" s="11" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="I20" s="11">
         <v>1.5770999999999999</v>
       </c>
       <c r="L20" s="6" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="M20" s="6" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="N20" s="6">
         <v>3.6</v>
@@ -4785,25 +6376,25 @@
     </row>
     <row r="21" spans="1:14" ht="13.15">
       <c r="B21" s="19" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="F21" s="11" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="G21" s="11" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="H21" s="11" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="I21" s="11">
         <v>1.5488</v>
       </c>
       <c r="L21" s="6" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="M21" s="6" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="N21" s="6">
         <v>1</v>
@@ -4811,25 +6402,25 @@
     </row>
     <row r="22" spans="1:14" ht="13.15">
       <c r="B22" s="19" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="F22" s="11" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="G22" s="11" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="H22" s="11" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="I22" s="11">
         <v>1.5224</v>
       </c>
       <c r="L22" s="6" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="M22" s="6" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="N22" s="6">
         <v>31.536000000000001</v>
@@ -4837,25 +6428,25 @@
     </row>
     <row r="23" spans="1:14" ht="13.15">
       <c r="B23" s="19" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="F23" s="11" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="G23" s="11" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="H23" s="11" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="I23" s="11">
         <v>1.5058</v>
       </c>
       <c r="L23" s="6" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="M23" s="6" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="N23" s="6">
         <v>120</v>
@@ -4863,25 +6454,25 @@
     </row>
     <row r="24" spans="1:14" ht="13.15">
       <c r="B24" s="19" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="F24" s="11" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="G24" s="11" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="H24" s="11" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="I24" s="11">
         <v>1.4844999999999999</v>
       </c>
       <c r="L24" s="11" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="M24" s="11" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="N24" s="11">
         <v>5.8615199999999996</v>
@@ -4889,25 +6480,25 @@
     </row>
     <row r="25" spans="1:14" ht="13.15">
       <c r="B25" s="19" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="F25" s="11" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="G25" s="11" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="H25" s="11" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="I25" s="11">
         <v>1.4518</v>
       </c>
       <c r="L25" s="11" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="M25" s="11" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="N25" s="11">
         <v>54</v>
@@ -4915,16 +6506,16 @@
     </row>
     <row r="26" spans="1:14" ht="13.15">
       <c r="B26" s="19" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="F26" s="11" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="G26" s="11" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="H26" s="11" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="I26" s="11">
         <v>1.4198999999999999</v>
@@ -4932,16 +6523,16 @@
     </row>
     <row r="27" spans="1:14" ht="13.15">
       <c r="B27" s="19" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="F27" s="11" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="G27" s="11" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="H27" s="11" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="I27" s="11">
         <v>1.3986000000000001</v>
@@ -4949,16 +6540,16 @@
     </row>
     <row r="28" spans="1:14" ht="13.15">
       <c r="B28" s="19" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="F28" s="11" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="G28" s="11" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="H28" s="11" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="I28" s="11">
         <v>1.3727</v>
@@ -4966,16 +6557,16 @@
     </row>
     <row r="29" spans="1:14" ht="13.15">
       <c r="B29" s="19" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="F29" s="11" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="G29" s="11" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="H29" s="11" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="I29" s="11">
         <v>1.3369</v>
@@ -4983,16 +6574,16 @@
     </row>
     <row r="30" spans="1:14" ht="13.15">
       <c r="B30" s="19" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="F30" s="11" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="G30" s="11" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="H30" s="11" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="I30" s="11">
         <v>1.2967</v>
@@ -5000,16 +6591,16 @@
     </row>
     <row r="31" spans="1:14" ht="13.15">
       <c r="B31" s="19" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="F31" s="11" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="G31" s="11" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="H31" s="11" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="I31" s="11">
         <v>1.2583</v>
@@ -5017,16 +6608,16 @@
     </row>
     <row r="32" spans="1:14" ht="13.15">
       <c r="B32" s="19" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="F32" s="11" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="G32" s="11" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="H32" s="11" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="I32" s="11">
         <v>1.2253000000000001</v>
@@ -5034,16 +6625,16 @@
     </row>
     <row r="33" spans="2:9" ht="13.15">
       <c r="B33" s="19" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="F33" s="11" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="G33" s="11" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="H33" s="11" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="I33" s="11">
         <v>1.2023999999999999</v>
@@ -5051,16 +6642,16 @@
     </row>
     <row r="34" spans="2:9" ht="13.15">
       <c r="B34" s="19" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="F34" s="11" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="G34" s="11" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="H34" s="11" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="I34" s="11">
         <v>1.1931</v>
@@ -5068,16 +6659,16 @@
     </row>
     <row r="35" spans="2:9" ht="13.15">
       <c r="B35" s="19" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="F35" s="11" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="G35" s="11" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="H35" s="11" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="I35" s="11">
         <v>1.1793</v>
@@ -5085,16 +6676,16 @@
     </row>
     <row r="36" spans="2:9" ht="13.15">
       <c r="B36" s="19" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="F36" s="11" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="G36" s="11" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="H36" s="11" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="I36" s="11">
         <v>1.1552</v>
@@ -5102,16 +6693,16 @@
     </row>
     <row r="37" spans="2:9" ht="13.15">
       <c r="B37" s="19" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="F37" s="11" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="G37" s="11" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="H37" s="11" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="I37" s="11">
         <v>1.1334</v>
@@ -5119,16 +6710,16 @@
     </row>
     <row r="38" spans="2:9" ht="13.15">
       <c r="B38" s="19" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="F38" s="11" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="G38" s="11" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="H38" s="11" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="I38" s="11">
         <v>1.1136999999999999</v>
@@ -5136,16 +6727,16 @@
     </row>
     <row r="39" spans="2:9" ht="13.15">
       <c r="B39" s="19" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="F39" s="11" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="G39" s="11" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="H39" s="11" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="I39" s="11">
         <v>1.0934999999999999</v>
@@ -5153,16 +6744,16 @@
     </row>
     <row r="40" spans="2:9" ht="13.15">
       <c r="B40" s="19" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="F40" s="11" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="G40" s="11" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="H40" s="11" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="I40" s="11">
         <v>1.0831</v>
@@ -5170,16 +6761,16 @@
     </row>
     <row r="41" spans="2:9" ht="13.15">
       <c r="B41" s="19" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="F41" s="11" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="G41" s="11" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="H41" s="11" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="I41" s="11">
         <v>1.0719000000000001</v>
@@ -5187,16 +6778,16 @@
     </row>
     <row r="42" spans="2:9" ht="13.15">
       <c r="B42" s="19" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="F42" s="11" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="G42" s="11" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="H42" s="11" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="I42" s="11">
         <v>1.0519000000000001</v>
@@ -5204,16 +6795,16 @@
     </row>
     <row r="43" spans="2:9" ht="13.15">
       <c r="B43" s="19" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="F43" s="11" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="G43" s="11" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="H43" s="11" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="I43" s="11">
         <v>1.0274000000000001</v>
@@ -5221,16 +6812,16 @@
     </row>
     <row r="44" spans="2:9" ht="13.15">
       <c r="B44" s="19" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="F44" s="11" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="G44" s="11" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="H44" s="11" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="I44" s="11">
         <v>1.0091000000000001</v>
@@ -5238,16 +6829,16 @@
     </row>
     <row r="45" spans="2:9" ht="13.15">
       <c r="B45" s="19" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="F45" s="11" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="G45" s="11" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="H45" s="11" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="I45" s="11">
         <v>1</v>
@@ -5255,16 +6846,16 @@
     </row>
     <row r="46" spans="2:9" ht="13.15">
       <c r="B46" s="19" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="F46" s="11" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="G46" s="11" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="H46" s="11" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="I46" s="11">
         <v>0.98960000000000004</v>
@@ -5272,16 +6863,16 @@
     </row>
     <row r="47" spans="2:9" ht="13.15">
       <c r="B47" s="19" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="F47" s="11" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="G47" s="11" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="H47" s="11" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="I47" s="11">
         <v>0.97809999999999997</v>
@@ -5289,16 +6880,16 @@
     </row>
     <row r="48" spans="2:9" ht="13.15">
       <c r="B48" s="19" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="F48" s="11" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="G48" s="11" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="H48" s="11" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="I48" s="11">
         <v>0.96499999999999997</v>
@@ -5306,16 +6897,16 @@
     </row>
     <row r="49" spans="2:9" ht="13.15">
       <c r="B49" s="19" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="F49" s="11" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="G49" s="11" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="H49" s="11" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="I49" s="11">
         <v>0.94910000000000005</v>
@@ -5323,16 +6914,16 @@
     </row>
     <row r="50" spans="2:9" ht="13.15">
       <c r="B50" s="19" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="F50" s="11" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="G50" s="11" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="H50" s="11" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="I50" s="11">
         <v>0.92969999999999997</v>
@@ -5340,7 +6931,7 @@
     </row>
     <row r="51" spans="2:9" ht="13.15">
       <c r="B51" s="19" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="F51" s="11" t="str">
         <f>F46</f>
@@ -5351,7 +6942,7 @@
         <v>USD20</v>
       </c>
       <c r="H51" s="11" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="I51" s="11">
         <f t="shared" si="0"/>
@@ -5360,13 +6951,13 @@
     </row>
     <row r="52" spans="2:9" ht="13.15">
       <c r="B52" s="19" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="F52" s="11" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="H52" s="11" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="I52" s="11">
         <v>7.0000000000000007E-2</v>
@@ -5374,13 +6965,13 @@
     </row>
     <row r="53" spans="2:9" ht="13.15">
       <c r="B53" s="19" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="F53" s="11" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="H53" s="11" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="I53" s="11">
         <v>7.0000000000000007E-2</v>
@@ -5388,13 +6979,13 @@
     </row>
     <row r="54" spans="2:9" ht="13.15">
       <c r="B54" s="19" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="F54" s="11" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="H54" s="11" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="I54" s="11">
         <v>7.0000000000000007E-2</v>
@@ -5402,10 +6993,10 @@
     </row>
     <row r="55" spans="2:9">
       <c r="F55" s="11" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="H55" s="11" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="I55" s="11">
         <v>7.0000000000000007E-2</v>
@@ -5413,10 +7004,10 @@
     </row>
     <row r="56" spans="2:9">
       <c r="F56" s="11" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="H56" s="11" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="I56" s="11">
         <v>7.0000000000000007E-2</v>
@@ -5424,10 +7015,10 @@
     </row>
     <row r="57" spans="2:9">
       <c r="F57" s="11" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="H57" s="11" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="I57" s="11">
         <v>7.0000000000000007E-2</v>
@@ -5435,10 +7026,10 @@
     </row>
     <row r="58" spans="2:9">
       <c r="F58" s="11" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="H58" s="11" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="I58" s="11">
         <v>7.0000000000000007E-2</v>
@@ -5446,10 +7037,10 @@
     </row>
     <row r="59" spans="2:9">
       <c r="F59" s="11" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="H59" s="11" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="I59" s="11">
         <v>7.0000000000000007E-2</v>
@@ -5457,10 +7048,10 @@
     </row>
     <row r="60" spans="2:9">
       <c r="F60" s="11" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="H60" s="11" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="I60" s="11">
         <v>7.0000000000000007E-2</v>
@@ -5468,10 +7059,10 @@
     </row>
     <row r="61" spans="2:9">
       <c r="F61" s="11" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="H61" s="11" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="I61" s="11">
         <v>7.0000000000000007E-2</v>
@@ -5479,10 +7070,10 @@
     </row>
     <row r="62" spans="2:9">
       <c r="F62" s="11" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="H62" s="11" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="I62" s="11">
         <v>7.0000000000000007E-2</v>
@@ -5490,10 +7081,10 @@
     </row>
     <row r="63" spans="2:9">
       <c r="F63" s="11" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="H63" s="11" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="I63" s="11">
         <v>7.0000000000000007E-2</v>
@@ -5501,10 +7092,10 @@
     </row>
     <row r="64" spans="2:9">
       <c r="F64" s="11" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="H64" s="11" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="I64" s="11">
         <v>7.0000000000000007E-2</v>
@@ -5512,10 +7103,10 @@
     </row>
     <row r="65" spans="6:9">
       <c r="F65" s="11" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="H65" s="11" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="I65" s="11">
         <v>7.0000000000000007E-2</v>
@@ -5523,10 +7114,10 @@
     </row>
     <row r="66" spans="6:9">
       <c r="F66" s="11" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="H66" s="11" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="I66" s="11">
         <v>7.0000000000000007E-2</v>
@@ -5534,10 +7125,10 @@
     </row>
     <row r="67" spans="6:9">
       <c r="F67" s="11" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="H67" s="11" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="I67" s="11">
         <v>7.0000000000000007E-2</v>
@@ -5545,10 +7136,10 @@
     </row>
     <row r="68" spans="6:9">
       <c r="F68" s="11" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="H68" s="11" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="I68" s="11">
         <v>7.0000000000000007E-2</v>
@@ -5556,10 +7147,10 @@
     </row>
     <row r="69" spans="6:9">
       <c r="F69" s="11" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="H69" s="11" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="I69" s="11">
         <v>7.0000000000000007E-2</v>
@@ -5567,10 +7158,10 @@
     </row>
     <row r="70" spans="6:9">
       <c r="F70" s="11" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="H70" s="11" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="I70" s="11">
         <v>7.0000000000000007E-2</v>
@@ -5578,10 +7169,10 @@
     </row>
     <row r="71" spans="6:9">
       <c r="F71" s="11" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="H71" s="11" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="I71" s="11">
         <v>7.0000000000000007E-2</v>
@@ -5589,10 +7180,10 @@
     </row>
     <row r="72" spans="6:9">
       <c r="F72" s="11" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="H72" s="11" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="I72" s="11">
         <v>7.0000000000000007E-2</v>
@@ -5600,10 +7191,10 @@
     </row>
     <row r="73" spans="6:9">
       <c r="F73" s="11" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="H73" s="11" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="I73" s="11">
         <v>7.0000000000000007E-2</v>
@@ -5611,10 +7202,10 @@
     </row>
     <row r="74" spans="6:9">
       <c r="F74" s="11" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="H74" s="11" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="I74" s="11">
         <v>7.0000000000000007E-2</v>
@@ -5622,10 +7213,10 @@
     </row>
     <row r="75" spans="6:9">
       <c r="F75" s="11" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="H75" s="11" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="I75" s="11">
         <v>7.0000000000000007E-2</v>
@@ -5633,10 +7224,10 @@
     </row>
     <row r="76" spans="6:9">
       <c r="F76" s="11" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="H76" s="11" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="I76" s="11">
         <v>7.0000000000000007E-2</v>
@@ -5644,10 +7235,10 @@
     </row>
     <row r="77" spans="6:9">
       <c r="F77" s="11" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="H77" s="11" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="I77" s="11">
         <v>7.0000000000000007E-2</v>
@@ -5655,10 +7246,10 @@
     </row>
     <row r="78" spans="6:9">
       <c r="F78" s="11" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="H78" s="11" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="I78" s="11">
         <v>7.0000000000000007E-2</v>
@@ -5666,10 +7257,10 @@
     </row>
     <row r="79" spans="6:9">
       <c r="F79" s="11" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="H79" s="11" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="I79" s="11">
         <v>7.0000000000000007E-2</v>
@@ -5677,10 +7268,10 @@
     </row>
     <row r="80" spans="6:9">
       <c r="F80" s="11" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="H80" s="11" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="I80" s="11">
         <v>7.0000000000000007E-2</v>
@@ -5688,10 +7279,10 @@
     </row>
     <row r="81" spans="6:9">
       <c r="F81" s="11" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="H81" s="11" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="I81" s="11">
         <v>7.0000000000000007E-2</v>
@@ -5699,10 +7290,10 @@
     </row>
     <row r="82" spans="6:9">
       <c r="F82" s="11" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="H82" s="11" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="I82" s="11">
         <v>7.0000000000000007E-2</v>
@@ -5710,10 +7301,10 @@
     </row>
     <row r="83" spans="6:9">
       <c r="F83" s="11" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="H83" s="11" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="I83" s="11">
         <v>7.0000000000000007E-2</v>
@@ -5721,10 +7312,10 @@
     </row>
     <row r="84" spans="6:9">
       <c r="F84" s="11" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="H84" s="11" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="I84" s="11">
         <v>7.0000000000000007E-2</v>
@@ -5732,10 +7323,10 @@
     </row>
     <row r="85" spans="6:9">
       <c r="F85" s="11" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="H85" s="11" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="I85" s="11">
         <v>7.0000000000000007E-2</v>
@@ -5743,10 +7334,10 @@
     </row>
     <row r="86" spans="6:9">
       <c r="F86" s="11" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="H86" s="11" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="I86" s="11">
         <v>7.0000000000000007E-2</v>
@@ -5754,10 +7345,10 @@
     </row>
     <row r="87" spans="6:9">
       <c r="F87" s="11" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="H87" s="11" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="I87" s="11">
         <v>7.0000000000000007E-2</v>
@@ -5765,10 +7356,10 @@
     </row>
     <row r="88" spans="6:9">
       <c r="F88" s="11" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="H88" s="11" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="I88" s="11">
         <v>7.0000000000000007E-2</v>
@@ -5776,10 +7367,10 @@
     </row>
     <row r="89" spans="6:9">
       <c r="F89" s="11" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="H89" s="11" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="I89" s="11">
         <v>7.0000000000000007E-2</v>
@@ -5787,10 +7378,10 @@
     </row>
     <row r="90" spans="6:9">
       <c r="F90" s="11" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="H90" s="11" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="I90" s="11">
         <v>7.0000000000000007E-2</v>
@@ -5798,10 +7389,10 @@
     </row>
     <row r="91" spans="6:9">
       <c r="F91" s="11" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="H91" s="11" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="I91" s="11">
         <v>7.0000000000000007E-2</v>
@@ -5809,10 +7400,10 @@
     </row>
     <row r="92" spans="6:9">
       <c r="F92" s="11" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="H92" s="11" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="I92" s="11">
         <v>7.0000000000000007E-2</v>
@@ -5820,10 +7411,10 @@
     </row>
     <row r="93" spans="6:9">
       <c r="F93" s="11" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="H93" s="11" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="I93" s="11">
         <v>7.0000000000000007E-2</v>
@@ -5831,10 +7422,10 @@
     </row>
     <row r="94" spans="6:9">
       <c r="F94" s="11" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="H94" s="11" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="I94" s="11">
         <v>7.0000000000000007E-2</v>
@@ -5842,7 +7433,7 @@
     </row>
     <row r="95" spans="6:9">
       <c r="F95" s="11" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="H95" s="11" t="str">
         <f>H51</f>
@@ -5854,39 +7445,39 @@
     </row>
     <row r="99" spans="5:10" ht="17.649999999999999" thickBot="1">
       <c r="E99" s="20" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
     </row>
     <row r="100" spans="5:10" ht="15" thickTop="1" thickBot="1">
       <c r="E100" s="4" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="F100" s="4" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="G100" s="4" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="H100" s="4" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="I100" s="4">
         <v>2022</v>
       </c>
       <c r="J100" s="4" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
     </row>
     <row r="101" spans="5:10" ht="14.25">
       <c r="E101"/>
       <c r="F101" s="21" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="G101" s="21" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="H101" s="21" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="I101" s="22">
         <f>1.10926234054354*I40</f>
@@ -5896,11 +7487,11 @@
     <row r="102" spans="5:10" ht="14.25">
       <c r="E102"/>
       <c r="F102" s="21" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="G102"/>
       <c r="H102" s="21" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="I102" s="22">
         <f>I84</f>
@@ -5925,26 +7516,26 @@
   <sheetData>
     <row r="3" spans="2:4" ht="17.649999999999999" thickBot="1">
       <c r="B3" s="20" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
     </row>
     <row r="4" spans="2:4" ht="15" thickTop="1" thickBot="1">
       <c r="B4" s="4" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="D4" s="4" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
     </row>
     <row r="5" spans="2:4">
       <c r="B5" s="6" t="s">
+        <v>154</v>
+      </c>
+      <c r="C5" s="6" t="s">
         <v>155</v>
-      </c>
-      <c r="C5" s="6" t="s">
-        <v>156</v>
       </c>
       <c r="D5" s="6">
         <v>-1</v>
@@ -5952,10 +7543,10 @@
     </row>
     <row r="6" spans="2:4">
       <c r="B6" s="6" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="C6" s="6" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="D6" s="6">
         <v>1</v>
@@ -5963,10 +7554,10 @@
     </row>
     <row r="7" spans="2:4">
       <c r="B7" s="6" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="C7" s="6" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="D7" s="6">
         <v>1</v>
@@ -5974,10 +7565,10 @@
     </row>
     <row r="8" spans="2:4">
       <c r="B8" s="6" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="C8" s="6" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="D8" s="6">
         <v>1</v>
@@ -5985,10 +7576,10 @@
     </row>
     <row r="9" spans="2:4">
       <c r="B9" s="6" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="C9" s="6" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="D9" s="6">
         <v>1</v>
@@ -5996,10 +7587,10 @@
     </row>
     <row r="10" spans="2:4">
       <c r="B10" s="6" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="C10" s="6" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="D10" s="6">
         <v>1</v>
@@ -6007,10 +7598,10 @@
     </row>
     <row r="11" spans="2:4">
       <c r="B11" s="6" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="C11" s="6" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="D11" s="6">
         <v>1</v>
@@ -6018,10 +7609,10 @@
     </row>
     <row r="12" spans="2:4">
       <c r="B12" s="6" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="C12" s="6" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="D12" s="6">
         <v>1</v>
@@ -6029,10 +7620,10 @@
     </row>
     <row r="13" spans="2:4">
       <c r="B13" s="6" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="C13" s="6" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="D13" s="6">
         <v>1</v>
@@ -6040,10 +7631,10 @@
     </row>
     <row r="14" spans="2:4">
       <c r="B14" s="6" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="C14" s="6" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="D14" s="6">
         <v>2</v>
@@ -6051,10 +7642,10 @@
     </row>
     <row r="15" spans="2:4">
       <c r="B15" s="6" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="C15" s="6" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="D15" s="6">
         <v>1</v>
@@ -6062,10 +7653,10 @@
     </row>
     <row r="16" spans="2:4">
       <c r="B16" s="6" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="C16" s="6" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="D16" s="16">
         <v>1.0000000000000001E-5</v>
@@ -6073,10 +7664,10 @@
     </row>
     <row r="17" spans="2:4">
       <c r="B17" s="6" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="C17" s="6" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="D17" s="16">
         <v>1.0000000000000001E-5</v>
@@ -6084,10 +7675,10 @@
     </row>
     <row r="18" spans="2:4">
       <c r="B18" s="6" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="C18" s="6" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="D18" s="16">
         <v>1.0000000000000001E-5</v>
@@ -6095,10 +7686,10 @@
     </row>
     <row r="19" spans="2:4">
       <c r="B19" s="6" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="C19" s="6" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="D19" s="16">
         <v>1.0000000000000001E-5</v>
@@ -6106,10 +7697,10 @@
     </row>
     <row r="20" spans="2:4">
       <c r="B20" s="6" t="s">
+        <v>169</v>
+      </c>
+      <c r="C20" s="6" t="s">
         <v>170</v>
-      </c>
-      <c r="C20" s="6" t="s">
-        <v>171</v>
       </c>
       <c r="D20" s="17">
         <v>1</v>
@@ -6117,73 +7708,73 @@
     </row>
     <row r="23" spans="2:4">
       <c r="B23" s="18" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
     </row>
     <row r="25" spans="2:4" ht="17.649999999999999" thickBot="1">
       <c r="B25" s="20" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
     </row>
     <row r="26" spans="2:4" ht="15" thickTop="1" thickBot="1">
       <c r="B26" s="4" t="s">
+        <v>173</v>
+      </c>
+      <c r="C26" s="4" t="s">
         <v>174</v>
-      </c>
-      <c r="C26" s="4" t="s">
-        <v>175</v>
       </c>
     </row>
     <row r="27" spans="2:4">
       <c r="B27" s="6" t="s">
+        <v>175</v>
+      </c>
+      <c r="C27" s="6" t="s">
         <v>176</v>
-      </c>
-      <c r="C27" s="6" t="s">
-        <v>177</v>
       </c>
     </row>
     <row r="28" spans="2:4">
       <c r="B28" s="6" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="C28" s="6" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
     </row>
     <row r="29" spans="2:4">
       <c r="B29" s="6" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="C29" s="6" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
     </row>
     <row r="30" spans="2:4">
       <c r="B30" s="6" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="C30" s="6" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
     </row>
     <row r="31" spans="2:4">
       <c r="B31" s="6" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="C31" s="6" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
     </row>
     <row r="32" spans="2:4">
       <c r="B32" s="6" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
     </row>
     <row r="33" spans="2:3">
       <c r="B33" s="6" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="C33" s="6" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
     </row>
   </sheetData>

</xml_diff>